<commit_message>
Use uppercase for PDB IDs
</commit_message>
<xml_diff>
--- a/Table S4 - PDB structures used for each virus.xlsx
+++ b/Table S4 - PDB structures used for each virus.xlsx
@@ -57,7 +57,7 @@
     <t xml:space="preserve">Obs.</t>
   </si>
   <si>
-    <t xml:space="preserve">5yxa</t>
+    <t xml:space="preserve">5YXA</t>
   </si>
   <si>
     <t xml:space="preserve">YFV</t>
@@ -66,31 +66,31 @@
     <t xml:space="preserve">C-terminal fragment only</t>
   </si>
   <si>
-    <t xml:space="preserve">8zba</t>
+    <t xml:space="preserve">8ZBA</t>
   </si>
   <si>
     <t xml:space="preserve">Tetrameric form</t>
   </si>
   <si>
-    <t xml:space="preserve">8zb9</t>
+    <t xml:space="preserve">8ZB9</t>
   </si>
   <si>
     <t xml:space="preserve">Dimeric form</t>
   </si>
   <si>
-    <t xml:space="preserve">7bsc</t>
+    <t xml:space="preserve">7BSC</t>
   </si>
   <si>
     <t xml:space="preserve">DENV2</t>
   </si>
   <si>
-    <t xml:space="preserve">7wus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7wut</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5k6k</t>
+    <t xml:space="preserve">7WUS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7WUT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5K6K</t>
   </si>
   <si>
     <t xml:space="preserve">ZIKV</t>

</xml_diff>